<commit_message>
Update game systems and cultivation rewards
</commit_message>
<xml_diff>
--- a/config/xlsx/initial_setup.xlsx
+++ b/config/xlsx/initial_setup.xlsx
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -791,69 +791,6 @@
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="n">
-        <v>12001</v>
-      </c>
-      <c r="C17" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="n">
-        <v>17001</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>main</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="n">
-        <v>16001</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>8</v>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>FALSE</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>